<commit_message>
Publish laneway-music record-company collection
</commit_message>
<xml_diff>
--- a/record-company-output/laneway-music/laneway-music-deep-cuts-report.xlsx
+++ b/record-company-output/laneway-music/laneway-music-deep-cuts-report.xlsx
@@ -456,14 +456,14 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>38</v>
+        <v>0</v>
       </c>
       <c r="B2" t="n">
         <v>57</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>laneway-music</t>
+          <t>Laneway Music</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -576,7 +576,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-07-25T03:28:06.329Z</t>
+          <t>2026-07-25T04:54:16.087Z</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -629,7 +629,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2026-07-25T03:28:06.475Z</t>
+          <t>2026-07-25T04:54:16.212Z</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -18185,7 +18185,7 @@
     <row r="218">
       <c r="B218" t="inlineStr">
         <is>
-          <t>2026-07-25T03:27:56.799Z</t>
+          <t>2026-07-25T04:54:03.765Z</t>
         </is>
       </c>
       <c r="C218" t="n">
@@ -18230,7 +18230,7 @@
     <row r="219">
       <c r="B219" t="inlineStr">
         <is>
-          <t>2026-07-25T03:27:56.799Z</t>
+          <t>2026-07-25T04:54:03.765Z</t>
         </is>
       </c>
       <c r="C219" t="n">
@@ -18248,7 +18248,7 @@
       </c>
       <c r="F219" t="inlineStr">
         <is>
-          <t>Official domain lanewaymusic.com.au identifies laneway-music.</t>
+          <t>Official domain lanewaymusic.com.au identifies Laneway Music.</t>
         </is>
       </c>
       <c r="G219" t="inlineStr">
@@ -18295,7 +18295,7 @@
     <col width="13" customWidth="1" min="7" max="7"/>
     <col width="55" customWidth="1" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
-    <col width="34" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
     <col width="15" customWidth="1" min="11" max="11"/>
     <col width="34" customWidth="1" min="12" max="12"/>
     <col width="19" customWidth="1" min="13" max="13"/>
@@ -18432,34 +18432,29 @@
           <t>https://static.wixstatic.com/media/9acc25_e7a33bd9f61f43bc96684220d1f0753f.png/v1/fit/w_2500,h_1330,al_c/9acc25_e7a33bd9f61f43bc96684220d1f0753f.png</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr">
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Laneway Music</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
         <is>
           <t>https://www.lanewaymusic.com.au/</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr">
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>rc_b9181116</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
         <is>
           <t>laneway-music</t>
         </is>
       </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>https://www.lanewaymusic.com.au/</t>
-        </is>
-      </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>rc_b9181116</t>
-        </is>
-      </c>
-      <c r="N2" t="inlineStr">
-        <is>
-          <t>laneway-music</t>
-        </is>
-      </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>[{"fieldName":"identity","sourceUrl":"https://www.lanewaymusic.com.au/","summary":"Official domain lanewaymusic.com.au identifies laneway-music.","confidenceScore":0.99,"checkedAt":"2026-07-25T03:27:56.799Z"},{"fieldName":"description","sourceUrl":"https://www.lanewaymusic.com.au/","summary":"Laneway Music distributes iconic artists catalogue digitally around the world.","confidenceScore":0.98,"checkedAt":"2026-07-25T03:27:56.799Z"}]</t>
+          <t>[{"fieldName":"identity","sourceUrl":"https://www.lanewaymusic.com.au/","summary":"Official domain lanewaymusic.com.au identifies Laneway Music.","confidenceScore":0.99,"checkedAt":"2026-07-25T04:54:03.765Z"},{"fieldName":"description","sourceUrl":"https://www.lanewaymusic.com.au/","summary":"Laneway Music distributes iconic artists catalogue digitally around the world.","confidenceScore":0.98,"checkedAt":"2026-07-25T04:54:03.765Z"}]</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
@@ -18469,7 +18464,7 @@
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>2026-07-25T04:12:00.557Z</t>
+          <t>2026-07-25T04:55:25.713Z</t>
         </is>
       </c>
     </row>
@@ -18653,7 +18648,7 @@
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>2026-07-25T03:29:01.589Z</t>
+          <t>2026-07-25T04:54:34.143Z</t>
         </is>
       </c>
     </row>
@@ -18713,7 +18708,7 @@
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>2026-07-25T03:29:12.278Z</t>
+          <t>2026-07-25T04:54:34.143Z</t>
         </is>
       </c>
     </row>
@@ -18773,7 +18768,7 @@
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t>2026-07-25T03:29:22.424Z</t>
+          <t>2026-07-25T04:54:34.143Z</t>
         </is>
       </c>
     </row>
@@ -18833,7 +18828,7 @@
       </c>
       <c r="P5" t="inlineStr">
         <is>
-          <t>2026-07-25T03:29:34.130Z</t>
+          <t>2026-07-25T04:54:34.143Z</t>
         </is>
       </c>
     </row>
@@ -18903,7 +18898,7 @@
       </c>
       <c r="P6" t="inlineStr">
         <is>
-          <t>2026-07-25T03:29:53.531Z</t>
+          <t>2026-07-25T04:54:34.143Z</t>
         </is>
       </c>
     </row>
@@ -18973,7 +18968,7 @@
       </c>
       <c r="P7" t="inlineStr">
         <is>
-          <t>2026-07-25T03:30:16.192Z</t>
+          <t>2026-07-25T04:54:34.143Z</t>
         </is>
       </c>
     </row>
@@ -19043,7 +19038,7 @@
       </c>
       <c r="P8" t="inlineStr">
         <is>
-          <t>2026-07-25T03:30:36.263Z</t>
+          <t>2026-07-25T04:54:34.143Z</t>
         </is>
       </c>
     </row>
@@ -19103,7 +19098,7 @@
       </c>
       <c r="P9" t="inlineStr">
         <is>
-          <t>2026-07-25T03:30:45.984Z</t>
+          <t>2026-07-25T04:54:34.143Z</t>
         </is>
       </c>
     </row>
@@ -19163,7 +19158,7 @@
       </c>
       <c r="P10" t="inlineStr">
         <is>
-          <t>2026-07-25T03:30:55.633Z</t>
+          <t>2026-07-25T04:54:34.143Z</t>
         </is>
       </c>
     </row>
@@ -19233,7 +19228,7 @@
       </c>
       <c r="P11" t="inlineStr">
         <is>
-          <t>2026-07-25T03:31:20.395Z</t>
+          <t>2026-07-25T04:54:34.143Z</t>
         </is>
       </c>
     </row>
@@ -19293,7 +19288,7 @@
       </c>
       <c r="P12" t="inlineStr">
         <is>
-          <t>2026-07-25T03:31:36.406Z</t>
+          <t>2026-07-25T04:54:34.143Z</t>
         </is>
       </c>
     </row>
@@ -19363,7 +19358,7 @@
       </c>
       <c r="P13" t="inlineStr">
         <is>
-          <t>2026-07-25T03:31:54.825Z</t>
+          <t>2026-07-25T04:54:34.143Z</t>
         </is>
       </c>
     </row>
@@ -19433,7 +19428,7 @@
       </c>
       <c r="P14" t="inlineStr">
         <is>
-          <t>2026-07-25T03:32:17.787Z</t>
+          <t>2026-07-25T04:54:34.143Z</t>
         </is>
       </c>
     </row>
@@ -19503,7 +19498,7 @@
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>2026-07-25T03:32:36.322Z</t>
+          <t>2026-07-25T04:54:34.143Z</t>
         </is>
       </c>
     </row>
@@ -19573,7 +19568,7 @@
       </c>
       <c r="P16" t="inlineStr">
         <is>
-          <t>2026-07-25T03:33:00.715Z</t>
+          <t>2026-07-25T04:54:34.143Z</t>
         </is>
       </c>
     </row>
@@ -19638,7 +19633,7 @@
       </c>
       <c r="P17" t="inlineStr">
         <is>
-          <t>2026-07-25T03:33:24.989Z</t>
+          <t>2026-07-25T04:54:34.143Z</t>
         </is>
       </c>
     </row>
@@ -19708,7 +19703,7 @@
       </c>
       <c r="P18" t="inlineStr">
         <is>
-          <t>2026-07-25T03:33:51.240Z</t>
+          <t>2026-07-25T04:54:34.143Z</t>
         </is>
       </c>
     </row>
@@ -19778,7 +19773,7 @@
       </c>
       <c r="P19" t="inlineStr">
         <is>
-          <t>2026-07-25T03:35:12.739Z</t>
+          <t>2026-07-25T04:54:34.143Z</t>
         </is>
       </c>
     </row>
@@ -19838,7 +19833,7 @@
       </c>
       <c r="P20" t="inlineStr">
         <is>
-          <t>2026-07-25T03:35:23.008Z</t>
+          <t>2026-07-25T04:54:34.143Z</t>
         </is>
       </c>
     </row>
@@ -19898,7 +19893,7 @@
       </c>
       <c r="P21" t="inlineStr">
         <is>
-          <t>2026-07-25T03:35:34.705Z</t>
+          <t>2026-07-25T04:54:34.143Z</t>
         </is>
       </c>
     </row>
@@ -19968,7 +19963,7 @@
       </c>
       <c r="P22" t="inlineStr">
         <is>
-          <t>2026-07-25T03:35:59.642Z</t>
+          <t>2026-07-25T04:54:34.143Z</t>
         </is>
       </c>
     </row>
@@ -20028,7 +20023,7 @@
       </c>
       <c r="P23" t="inlineStr">
         <is>
-          <t>2026-07-25T03:36:10.070Z</t>
+          <t>2026-07-25T04:54:34.143Z</t>
         </is>
       </c>
     </row>
@@ -20098,7 +20093,7 @@
       </c>
       <c r="P24" t="inlineStr">
         <is>
-          <t>2026-07-25T03:36:31.594Z</t>
+          <t>2026-07-25T04:54:34.143Z</t>
         </is>
       </c>
     </row>
@@ -20158,7 +20153,7 @@
       </c>
       <c r="P25" t="inlineStr">
         <is>
-          <t>2026-07-25T03:36:43.976Z</t>
+          <t>2026-07-25T04:54:34.143Z</t>
         </is>
       </c>
     </row>
@@ -20228,7 +20223,7 @@
       </c>
       <c r="P26" t="inlineStr">
         <is>
-          <t>2026-07-25T03:37:02.827Z</t>
+          <t>2026-07-25T04:54:34.143Z</t>
         </is>
       </c>
     </row>
@@ -20288,7 +20283,7 @@
       </c>
       <c r="P27" t="inlineStr">
         <is>
-          <t>2026-07-25T03:37:12.313Z</t>
+          <t>2026-07-25T04:54:34.143Z</t>
         </is>
       </c>
     </row>
@@ -20358,7 +20353,7 @@
       </c>
       <c r="P28" t="inlineStr">
         <is>
-          <t>2026-07-25T03:37:31.061Z</t>
+          <t>2026-07-25T04:54:34.143Z</t>
         </is>
       </c>
     </row>
@@ -20418,7 +20413,7 @@
       </c>
       <c r="P29" t="inlineStr">
         <is>
-          <t>2026-07-25T03:37:43.747Z</t>
+          <t>2026-07-25T04:54:34.143Z</t>
         </is>
       </c>
     </row>
@@ -20488,7 +20483,7 @@
       </c>
       <c r="P30" t="inlineStr">
         <is>
-          <t>2026-07-25T03:38:03.302Z</t>
+          <t>2026-07-25T04:54:34.143Z</t>
         </is>
       </c>
     </row>
@@ -20548,7 +20543,7 @@
       </c>
       <c r="P31" t="inlineStr">
         <is>
-          <t>2026-07-25T03:38:14.017Z</t>
+          <t>2026-07-25T04:54:34.143Z</t>
         </is>
       </c>
     </row>
@@ -20613,7 +20608,7 @@
       </c>
       <c r="P32" t="inlineStr">
         <is>
-          <t>2026-07-25T03:38:39.774Z</t>
+          <t>2026-07-25T04:54:34.143Z</t>
         </is>
       </c>
     </row>
@@ -20673,7 +20668,7 @@
       </c>
       <c r="P33" t="inlineStr">
         <is>
-          <t>2026-07-25T03:38:59.457Z</t>
+          <t>2026-07-25T04:54:34.143Z</t>
         </is>
       </c>
     </row>
@@ -20743,7 +20738,7 @@
       </c>
       <c r="P34" t="inlineStr">
         <is>
-          <t>2026-07-25T03:39:29.064Z</t>
+          <t>2026-07-25T04:54:34.143Z</t>
         </is>
       </c>
     </row>
@@ -20803,7 +20798,7 @@
       </c>
       <c r="P35" t="inlineStr">
         <is>
-          <t>2026-07-25T03:39:50.126Z</t>
+          <t>2026-07-25T04:54:34.143Z</t>
         </is>
       </c>
     </row>
@@ -20863,7 +20858,7 @@
       </c>
       <c r="P36" t="inlineStr">
         <is>
-          <t>2026-07-25T03:40:07.793Z</t>
+          <t>2026-07-25T04:54:34.143Z</t>
         </is>
       </c>
     </row>
@@ -20933,7 +20928,7 @@
       </c>
       <c r="P37" t="inlineStr">
         <is>
-          <t>2026-07-25T03:40:36.270Z</t>
+          <t>2026-07-25T04:54:34.143Z</t>
         </is>
       </c>
     </row>
@@ -21003,7 +20998,7 @@
       </c>
       <c r="P38" t="inlineStr">
         <is>
-          <t>2026-07-25T03:40:58.312Z</t>
+          <t>2026-07-25T04:54:34.143Z</t>
         </is>
       </c>
     </row>
@@ -21063,7 +21058,7 @@
       </c>
       <c r="P39" t="inlineStr">
         <is>
-          <t>2026-07-25T03:41:09.847Z</t>
+          <t>2026-07-25T04:54:34.143Z</t>
         </is>
       </c>
     </row>
@@ -21133,7 +21128,7 @@
       </c>
       <c r="P40" t="inlineStr">
         <is>
-          <t>2026-07-25T03:41:34.801Z</t>
+          <t>2026-07-25T04:54:34.143Z</t>
         </is>
       </c>
     </row>
@@ -21203,7 +21198,7 @@
       </c>
       <c r="P41" t="inlineStr">
         <is>
-          <t>2026-07-25T03:42:03.529Z</t>
+          <t>2026-07-25T04:54:34.143Z</t>
         </is>
       </c>
     </row>
@@ -21273,7 +21268,7 @@
       </c>
       <c r="P42" t="inlineStr">
         <is>
-          <t>2026-07-25T03:42:31.608Z</t>
+          <t>2026-07-25T04:54:34.143Z</t>
         </is>
       </c>
     </row>
@@ -21333,7 +21328,7 @@
       </c>
       <c r="P43" t="inlineStr">
         <is>
-          <t>2026-07-25T03:42:44.368Z</t>
+          <t>2026-07-25T04:54:34.143Z</t>
         </is>
       </c>
     </row>
@@ -21403,7 +21398,7 @@
       </c>
       <c r="P44" t="inlineStr">
         <is>
-          <t>2026-07-25T03:43:18.478Z</t>
+          <t>2026-07-25T04:54:34.143Z</t>
         </is>
       </c>
     </row>
@@ -21463,7 +21458,7 @@
       </c>
       <c r="P45" t="inlineStr">
         <is>
-          <t>2026-07-25T03:43:34.066Z</t>
+          <t>2026-07-25T04:54:34.143Z</t>
         </is>
       </c>
     </row>
@@ -21533,7 +21528,7 @@
       </c>
       <c r="P46" t="inlineStr">
         <is>
-          <t>2026-07-25T03:44:07.776Z</t>
+          <t>2026-07-25T04:54:34.143Z</t>
         </is>
       </c>
     </row>
@@ -21593,7 +21588,7 @@
       </c>
       <c r="P47" t="inlineStr">
         <is>
-          <t>2026-07-25T03:44:20.767Z</t>
+          <t>2026-07-25T04:54:34.143Z</t>
         </is>
       </c>
     </row>
@@ -21658,7 +21653,7 @@
       </c>
       <c r="P48" t="inlineStr">
         <is>
-          <t>2026-07-25T03:44:45.974Z</t>
+          <t>2026-07-25T04:54:34.143Z</t>
         </is>
       </c>
     </row>
@@ -21728,7 +21723,7 @@
       </c>
       <c r="P49" t="inlineStr">
         <is>
-          <t>2026-07-25T03:45:20.100Z</t>
+          <t>2026-07-25T04:54:34.143Z</t>
         </is>
       </c>
     </row>
@@ -21798,7 +21793,7 @@
       </c>
       <c r="P50" t="inlineStr">
         <is>
-          <t>2026-07-25T03:45:42.358Z</t>
+          <t>2026-07-25T04:54:34.143Z</t>
         </is>
       </c>
     </row>
@@ -21868,7 +21863,7 @@
       </c>
       <c r="P51" t="inlineStr">
         <is>
-          <t>2026-07-25T03:46:04.035Z</t>
+          <t>2026-07-25T04:54:34.143Z</t>
         </is>
       </c>
     </row>
@@ -21938,7 +21933,7 @@
       </c>
       <c r="P52" t="inlineStr">
         <is>
-          <t>2026-07-25T03:46:26.880Z</t>
+          <t>2026-07-25T04:54:34.143Z</t>
         </is>
       </c>
     </row>
@@ -22008,7 +22003,7 @@
       </c>
       <c r="P53" t="inlineStr">
         <is>
-          <t>2026-07-25T03:46:57.392Z</t>
+          <t>2026-07-25T04:54:34.143Z</t>
         </is>
       </c>
     </row>
@@ -22078,7 +22073,7 @@
       </c>
       <c r="P54" t="inlineStr">
         <is>
-          <t>2026-07-25T03:47:34.160Z</t>
+          <t>2026-07-25T04:54:34.143Z</t>
         </is>
       </c>
     </row>
@@ -22148,7 +22143,7 @@
       </c>
       <c r="P55" t="inlineStr">
         <is>
-          <t>2026-07-25T03:47:55.372Z</t>
+          <t>2026-07-25T04:54:34.143Z</t>
         </is>
       </c>
     </row>
@@ -22218,7 +22213,7 @@
       </c>
       <c r="P56" t="inlineStr">
         <is>
-          <t>2026-07-25T03:48:13.993Z</t>
+          <t>2026-07-25T04:54:34.143Z</t>
         </is>
       </c>
     </row>
@@ -22288,7 +22283,7 @@
       </c>
       <c r="P57" t="inlineStr">
         <is>
-          <t>2026-07-25T03:48:35.576Z</t>
+          <t>2026-07-25T04:54:34.143Z</t>
         </is>
       </c>
     </row>
@@ -22353,7 +22348,7 @@
       </c>
       <c r="P58" t="inlineStr">
         <is>
-          <t>2026-07-25T03:48:54.981Z</t>
+          <t>2026-07-25T04:54:34.143Z</t>
         </is>
       </c>
     </row>
@@ -22413,7 +22408,7 @@
       </c>
       <c r="P59" t="inlineStr">
         <is>
-          <t>2026-07-25T03:49:08.889Z</t>
+          <t>2026-07-25T04:54:34.143Z</t>
         </is>
       </c>
     </row>
@@ -22473,7 +22468,7 @@
       </c>
       <c r="P60" t="inlineStr">
         <is>
-          <t>2026-07-25T03:49:19.951Z</t>
+          <t>2026-07-25T04:54:34.143Z</t>
         </is>
       </c>
     </row>
@@ -22543,7 +22538,7 @@
       </c>
       <c r="P61" t="inlineStr">
         <is>
-          <t>2026-07-25T03:49:36.427Z</t>
+          <t>2026-07-25T04:54:34.143Z</t>
         </is>
       </c>
     </row>
@@ -22603,7 +22598,7 @@
       </c>
       <c r="P62" t="inlineStr">
         <is>
-          <t>2026-07-25T03:49:47.549Z</t>
+          <t>2026-07-25T04:54:34.143Z</t>
         </is>
       </c>
     </row>
@@ -22663,7 +22658,7 @@
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>2026-07-25T03:49:56.866Z</t>
+          <t>2026-07-25T04:54:34.143Z</t>
         </is>
       </c>
     </row>
@@ -22733,7 +22728,7 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>2026-07-25T03:50:17.369Z</t>
+          <t>2026-07-25T04:54:34.143Z</t>
         </is>
       </c>
     </row>
@@ -22803,7 +22798,7 @@
       </c>
       <c r="P65" t="inlineStr">
         <is>
-          <t>2026-07-25T03:50:39.891Z</t>
+          <t>2026-07-25T04:54:34.143Z</t>
         </is>
       </c>
     </row>
@@ -22863,7 +22858,7 @@
       </c>
       <c r="P66" t="inlineStr">
         <is>
-          <t>2026-07-25T03:50:49.246Z</t>
+          <t>2026-07-25T04:54:34.143Z</t>
         </is>
       </c>
     </row>
@@ -22933,7 +22928,7 @@
       </c>
       <c r="P67" t="inlineStr">
         <is>
-          <t>2026-07-25T03:54:37.637Z</t>
+          <t>2026-07-25T04:54:34.143Z</t>
         </is>
       </c>
     </row>
@@ -22993,7 +22988,7 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>2026-07-25T03:54:54.727Z</t>
+          <t>2026-07-25T04:54:34.143Z</t>
         </is>
       </c>
     </row>
@@ -23053,7 +23048,7 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>2026-07-25T03:55:05.884Z</t>
+          <t>2026-07-25T04:54:34.143Z</t>
         </is>
       </c>
     </row>
@@ -23123,7 +23118,7 @@
       </c>
       <c r="P70" t="inlineStr">
         <is>
-          <t>2026-07-25T03:55:25.890Z</t>
+          <t>2026-07-25T04:54:34.143Z</t>
         </is>
       </c>
     </row>
@@ -23183,7 +23178,7 @@
       </c>
       <c r="P71" t="inlineStr">
         <is>
-          <t>2026-07-25T03:55:35.222Z</t>
+          <t>2026-07-25T04:54:34.143Z</t>
         </is>
       </c>
     </row>
@@ -23253,7 +23248,7 @@
       </c>
       <c r="P72" t="inlineStr">
         <is>
-          <t>2026-07-25T03:55:52.740Z</t>
+          <t>2026-07-25T04:54:34.143Z</t>
         </is>
       </c>
     </row>
@@ -23313,7 +23308,7 @@
       </c>
       <c r="P73" t="inlineStr">
         <is>
-          <t>2026-07-25T03:56:07.707Z</t>
+          <t>2026-07-25T04:54:34.143Z</t>
         </is>
       </c>
     </row>
@@ -23378,7 +23373,7 @@
       </c>
       <c r="P74" t="inlineStr">
         <is>
-          <t>2026-07-25T03:56:26.212Z</t>
+          <t>2026-07-25T04:54:34.143Z</t>
         </is>
       </c>
     </row>
@@ -23443,7 +23438,7 @@
       </c>
       <c r="P75" t="inlineStr">
         <is>
-          <t>2026-07-25T03:56:46.139Z</t>
+          <t>2026-07-25T04:54:34.143Z</t>
         </is>
       </c>
     </row>
@@ -23513,7 +23508,7 @@
       </c>
       <c r="P76" t="inlineStr">
         <is>
-          <t>2026-07-25T03:57:12.330Z</t>
+          <t>2026-07-25T04:54:34.143Z</t>
         </is>
       </c>
     </row>
@@ -23583,7 +23578,7 @@
       </c>
       <c r="P77" t="inlineStr">
         <is>
-          <t>2026-07-25T03:57:37.841Z</t>
+          <t>2026-07-25T04:54:34.143Z</t>
         </is>
       </c>
     </row>
@@ -23643,7 +23638,7 @@
       </c>
       <c r="P78" t="inlineStr">
         <is>
-          <t>2026-07-25T03:57:46.784Z</t>
+          <t>2026-07-25T04:54:34.143Z</t>
         </is>
       </c>
     </row>
@@ -23703,7 +23698,7 @@
       </c>
       <c r="P79" t="inlineStr">
         <is>
-          <t>2026-07-25T03:57:58.984Z</t>
+          <t>2026-07-25T04:54:34.143Z</t>
         </is>
       </c>
     </row>
@@ -23763,7 +23758,7 @@
       </c>
       <c r="P80" t="inlineStr">
         <is>
-          <t>2026-07-25T03:58:08.835Z</t>
+          <t>2026-07-25T04:54:34.143Z</t>
         </is>
       </c>
     </row>
@@ -23828,7 +23823,7 @@
       </c>
       <c r="P81" t="inlineStr">
         <is>
-          <t>2026-07-25T04:04:26.310Z</t>
+          <t>2026-07-25T04:54:34.143Z</t>
         </is>
       </c>
     </row>
@@ -23898,7 +23893,7 @@
       </c>
       <c r="P82" t="inlineStr">
         <is>
-          <t>2026-07-25T04:04:50.280Z</t>
+          <t>2026-07-25T04:54:34.143Z</t>
         </is>
       </c>
     </row>
@@ -23958,7 +23953,7 @@
       </c>
       <c r="P83" t="inlineStr">
         <is>
-          <t>2026-07-25T04:05:09.082Z</t>
+          <t>2026-07-25T04:54:34.143Z</t>
         </is>
       </c>
     </row>
@@ -24028,7 +24023,7 @@
       </c>
       <c r="P84" t="inlineStr">
         <is>
-          <t>2026-07-25T04:05:31.707Z</t>
+          <t>2026-07-25T04:54:34.143Z</t>
         </is>
       </c>
     </row>
@@ -24093,7 +24088,7 @@
       </c>
       <c r="P85" t="inlineStr">
         <is>
-          <t>2026-07-25T04:06:06.428Z</t>
+          <t>2026-07-25T04:54:34.143Z</t>
         </is>
       </c>
     </row>
@@ -24153,7 +24148,7 @@
       </c>
       <c r="P86" t="inlineStr">
         <is>
-          <t>2026-07-25T04:06:20.312Z</t>
+          <t>2026-07-25T04:54:34.143Z</t>
         </is>
       </c>
     </row>
@@ -24223,7 +24218,7 @@
       </c>
       <c r="P87" t="inlineStr">
         <is>
-          <t>2026-07-25T04:06:38.630Z</t>
+          <t>2026-07-25T04:54:34.143Z</t>
         </is>
       </c>
     </row>
@@ -24293,7 +24288,7 @@
       </c>
       <c r="P88" t="inlineStr">
         <is>
-          <t>2026-07-25T04:06:58.252Z</t>
+          <t>2026-07-25T04:54:34.143Z</t>
         </is>
       </c>
     </row>
@@ -24363,7 +24358,7 @@
       </c>
       <c r="P89" t="inlineStr">
         <is>
-          <t>2026-07-25T04:07:19.046Z</t>
+          <t>2026-07-25T04:54:34.143Z</t>
         </is>
       </c>
     </row>
@@ -24423,7 +24418,7 @@
       </c>
       <c r="P90" t="inlineStr">
         <is>
-          <t>2026-07-25T04:07:30.042Z</t>
+          <t>2026-07-25T04:54:34.143Z</t>
         </is>
       </c>
     </row>
@@ -24483,7 +24478,7 @@
       </c>
       <c r="P91" t="inlineStr">
         <is>
-          <t>2026-07-25T04:07:40.743Z</t>
+          <t>2026-07-25T04:54:34.143Z</t>
         </is>
       </c>
     </row>
@@ -24553,7 +24548,7 @@
       </c>
       <c r="P92" t="inlineStr">
         <is>
-          <t>2026-07-25T04:08:10.250Z</t>
+          <t>2026-07-25T04:54:34.143Z</t>
         </is>
       </c>
     </row>
@@ -24613,7 +24608,7 @@
       </c>
       <c r="P93" t="inlineStr">
         <is>
-          <t>2026-07-25T04:08:23.673Z</t>
+          <t>2026-07-25T04:54:34.143Z</t>
         </is>
       </c>
     </row>
@@ -24683,7 +24678,7 @@
       </c>
       <c r="P94" t="inlineStr">
         <is>
-          <t>2026-07-25T04:10:35.995Z</t>
+          <t>2026-07-25T04:54:34.143Z</t>
         </is>
       </c>
     </row>
@@ -24753,7 +24748,7 @@
       </c>
       <c r="P95" t="inlineStr">
         <is>
-          <t>2026-07-25T04:11:17.108Z</t>
+          <t>2026-07-25T04:54:34.143Z</t>
         </is>
       </c>
     </row>
@@ -24813,7 +24808,7 @@
       </c>
       <c r="P96" t="inlineStr">
         <is>
-          <t>2026-07-25T04:11:34.428Z</t>
+          <t>2026-07-25T04:54:34.143Z</t>
         </is>
       </c>
     </row>
@@ -24997,7 +24992,7 @@
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>2026-07-25T03:29:01.589Z</t>
+          <t>2026-07-25T04:54:34.143Z</t>
         </is>
       </c>
     </row>
@@ -25067,7 +25062,7 @@
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>2026-07-25T03:29:53.531Z</t>
+          <t>2026-07-25T04:54:34.143Z</t>
         </is>
       </c>
     </row>
@@ -25137,7 +25132,7 @@
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t>2026-07-25T03:30:16.192Z</t>
+          <t>2026-07-25T04:54:34.143Z</t>
         </is>
       </c>
     </row>
@@ -25207,7 +25202,7 @@
       </c>
       <c r="P5" t="inlineStr">
         <is>
-          <t>2026-07-25T03:30:36.263Z</t>
+          <t>2026-07-25T04:54:34.143Z</t>
         </is>
       </c>
     </row>
@@ -25277,7 +25272,7 @@
       </c>
       <c r="P6" t="inlineStr">
         <is>
-          <t>2026-07-25T03:31:20.395Z</t>
+          <t>2026-07-25T04:54:34.143Z</t>
         </is>
       </c>
     </row>
@@ -25347,7 +25342,7 @@
       </c>
       <c r="P7" t="inlineStr">
         <is>
-          <t>2026-07-25T03:31:54.825Z</t>
+          <t>2026-07-25T04:54:34.143Z</t>
         </is>
       </c>
     </row>
@@ -25417,7 +25412,7 @@
       </c>
       <c r="P8" t="inlineStr">
         <is>
-          <t>2026-07-25T03:32:17.787Z</t>
+          <t>2026-07-25T04:54:34.143Z</t>
         </is>
       </c>
     </row>
@@ -25487,7 +25482,7 @@
       </c>
       <c r="P9" t="inlineStr">
         <is>
-          <t>2026-07-25T03:32:36.322Z</t>
+          <t>2026-07-25T04:54:34.143Z</t>
         </is>
       </c>
     </row>
@@ -25557,7 +25552,7 @@
       </c>
       <c r="P10" t="inlineStr">
         <is>
-          <t>2026-07-25T03:33:00.715Z</t>
+          <t>2026-07-25T04:54:34.143Z</t>
         </is>
       </c>
     </row>
@@ -25622,7 +25617,7 @@
       </c>
       <c r="P11" t="inlineStr">
         <is>
-          <t>2026-07-25T03:33:24.989Z</t>
+          <t>2026-07-25T04:54:34.143Z</t>
         </is>
       </c>
     </row>
@@ -25692,7 +25687,7 @@
       </c>
       <c r="P12" t="inlineStr">
         <is>
-          <t>2026-07-25T03:33:51.240Z</t>
+          <t>2026-07-25T04:54:34.143Z</t>
         </is>
       </c>
     </row>
@@ -25762,7 +25757,7 @@
       </c>
       <c r="P13" t="inlineStr">
         <is>
-          <t>2026-07-25T03:35:12.739Z</t>
+          <t>2026-07-25T04:54:34.143Z</t>
         </is>
       </c>
     </row>
@@ -25832,7 +25827,7 @@
       </c>
       <c r="P14" t="inlineStr">
         <is>
-          <t>2026-07-25T03:35:59.642Z</t>
+          <t>2026-07-25T04:54:34.143Z</t>
         </is>
       </c>
     </row>
@@ -25902,7 +25897,7 @@
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>2026-07-25T03:36:31.594Z</t>
+          <t>2026-07-25T04:54:34.143Z</t>
         </is>
       </c>
     </row>
@@ -25972,7 +25967,7 @@
       </c>
       <c r="P16" t="inlineStr">
         <is>
-          <t>2026-07-25T03:37:02.827Z</t>
+          <t>2026-07-25T04:54:34.143Z</t>
         </is>
       </c>
     </row>
@@ -26042,7 +26037,7 @@
       </c>
       <c r="P17" t="inlineStr">
         <is>
-          <t>2026-07-25T03:37:31.061Z</t>
+          <t>2026-07-25T04:54:34.143Z</t>
         </is>
       </c>
     </row>
@@ -26112,7 +26107,7 @@
       </c>
       <c r="P18" t="inlineStr">
         <is>
-          <t>2026-07-25T03:38:03.302Z</t>
+          <t>2026-07-25T04:54:34.143Z</t>
         </is>
       </c>
     </row>
@@ -26177,7 +26172,7 @@
       </c>
       <c r="P19" t="inlineStr">
         <is>
-          <t>2026-07-25T03:38:39.774Z</t>
+          <t>2026-07-25T04:54:34.143Z</t>
         </is>
       </c>
     </row>
@@ -26247,7 +26242,7 @@
       </c>
       <c r="P20" t="inlineStr">
         <is>
-          <t>2026-07-25T03:39:29.064Z</t>
+          <t>2026-07-25T04:54:34.143Z</t>
         </is>
       </c>
     </row>
@@ -26317,7 +26312,7 @@
       </c>
       <c r="P21" t="inlineStr">
         <is>
-          <t>2026-07-25T03:40:36.270Z</t>
+          <t>2026-07-25T04:54:34.143Z</t>
         </is>
       </c>
     </row>
@@ -26387,7 +26382,7 @@
       </c>
       <c r="P22" t="inlineStr">
         <is>
-          <t>2026-07-25T03:40:58.312Z</t>
+          <t>2026-07-25T04:54:34.143Z</t>
         </is>
       </c>
     </row>
@@ -26457,7 +26452,7 @@
       </c>
       <c r="P23" t="inlineStr">
         <is>
-          <t>2026-07-25T03:41:34.801Z</t>
+          <t>2026-07-25T04:54:34.143Z</t>
         </is>
       </c>
     </row>
@@ -26527,7 +26522,7 @@
       </c>
       <c r="P24" t="inlineStr">
         <is>
-          <t>2026-07-25T03:42:03.529Z</t>
+          <t>2026-07-25T04:54:34.143Z</t>
         </is>
       </c>
     </row>
@@ -26597,7 +26592,7 @@
       </c>
       <c r="P25" t="inlineStr">
         <is>
-          <t>2026-07-25T03:42:31.608Z</t>
+          <t>2026-07-25T04:54:34.143Z</t>
         </is>
       </c>
     </row>
@@ -26667,7 +26662,7 @@
       </c>
       <c r="P26" t="inlineStr">
         <is>
-          <t>2026-07-25T03:43:18.478Z</t>
+          <t>2026-07-25T04:54:34.143Z</t>
         </is>
       </c>
     </row>
@@ -26737,7 +26732,7 @@
       </c>
       <c r="P27" t="inlineStr">
         <is>
-          <t>2026-07-25T03:44:07.776Z</t>
+          <t>2026-07-25T04:54:34.143Z</t>
         </is>
       </c>
     </row>
@@ -26802,7 +26797,7 @@
       </c>
       <c r="P28" t="inlineStr">
         <is>
-          <t>2026-07-25T03:44:45.974Z</t>
+          <t>2026-07-25T04:54:34.143Z</t>
         </is>
       </c>
     </row>
@@ -26872,7 +26867,7 @@
       </c>
       <c r="P29" t="inlineStr">
         <is>
-          <t>2026-07-25T03:45:20.100Z</t>
+          <t>2026-07-25T04:54:34.143Z</t>
         </is>
       </c>
     </row>
@@ -26942,7 +26937,7 @@
       </c>
       <c r="P30" t="inlineStr">
         <is>
-          <t>2026-07-25T03:45:42.358Z</t>
+          <t>2026-07-25T04:54:34.143Z</t>
         </is>
       </c>
     </row>
@@ -27012,7 +27007,7 @@
       </c>
       <c r="P31" t="inlineStr">
         <is>
-          <t>2026-07-25T03:46:04.035Z</t>
+          <t>2026-07-25T04:54:34.143Z</t>
         </is>
       </c>
     </row>
@@ -27082,7 +27077,7 @@
       </c>
       <c r="P32" t="inlineStr">
         <is>
-          <t>2026-07-25T03:46:26.880Z</t>
+          <t>2026-07-25T04:54:34.143Z</t>
         </is>
       </c>
     </row>
@@ -27152,7 +27147,7 @@
       </c>
       <c r="P33" t="inlineStr">
         <is>
-          <t>2026-07-25T03:46:57.392Z</t>
+          <t>2026-07-25T04:54:34.143Z</t>
         </is>
       </c>
     </row>
@@ -27222,7 +27217,7 @@
       </c>
       <c r="P34" t="inlineStr">
         <is>
-          <t>2026-07-25T03:47:34.160Z</t>
+          <t>2026-07-25T04:54:34.143Z</t>
         </is>
       </c>
     </row>
@@ -27292,7 +27287,7 @@
       </c>
       <c r="P35" t="inlineStr">
         <is>
-          <t>2026-07-25T03:47:55.372Z</t>
+          <t>2026-07-25T04:54:34.143Z</t>
         </is>
       </c>
     </row>
@@ -27362,7 +27357,7 @@
       </c>
       <c r="P36" t="inlineStr">
         <is>
-          <t>2026-07-25T03:48:13.993Z</t>
+          <t>2026-07-25T04:54:34.143Z</t>
         </is>
       </c>
     </row>
@@ -27432,7 +27427,7 @@
       </c>
       <c r="P37" t="inlineStr">
         <is>
-          <t>2026-07-25T03:48:35.576Z</t>
+          <t>2026-07-25T04:54:34.143Z</t>
         </is>
       </c>
     </row>
@@ -27497,7 +27492,7 @@
       </c>
       <c r="P38" t="inlineStr">
         <is>
-          <t>2026-07-25T03:48:54.981Z</t>
+          <t>2026-07-25T04:54:34.143Z</t>
         </is>
       </c>
     </row>
@@ -27567,7 +27562,7 @@
       </c>
       <c r="P39" t="inlineStr">
         <is>
-          <t>2026-07-25T03:49:36.427Z</t>
+          <t>2026-07-25T04:54:34.143Z</t>
         </is>
       </c>
     </row>
@@ -27637,7 +27632,7 @@
       </c>
       <c r="P40" t="inlineStr">
         <is>
-          <t>2026-07-25T03:50:17.369Z</t>
+          <t>2026-07-25T04:54:34.143Z</t>
         </is>
       </c>
     </row>
@@ -27707,7 +27702,7 @@
       </c>
       <c r="P41" t="inlineStr">
         <is>
-          <t>2026-07-25T03:50:39.891Z</t>
+          <t>2026-07-25T04:54:34.143Z</t>
         </is>
       </c>
     </row>
@@ -27777,7 +27772,7 @@
       </c>
       <c r="P42" t="inlineStr">
         <is>
-          <t>2026-07-25T03:54:37.637Z</t>
+          <t>2026-07-25T04:54:34.143Z</t>
         </is>
       </c>
     </row>
@@ -27847,7 +27842,7 @@
       </c>
       <c r="P43" t="inlineStr">
         <is>
-          <t>2026-07-25T03:55:25.890Z</t>
+          <t>2026-07-25T04:54:34.143Z</t>
         </is>
       </c>
     </row>
@@ -27917,7 +27912,7 @@
       </c>
       <c r="P44" t="inlineStr">
         <is>
-          <t>2026-07-25T03:55:52.740Z</t>
+          <t>2026-07-25T04:54:34.143Z</t>
         </is>
       </c>
     </row>
@@ -27982,7 +27977,7 @@
       </c>
       <c r="P45" t="inlineStr">
         <is>
-          <t>2026-07-25T03:56:26.212Z</t>
+          <t>2026-07-25T04:54:34.143Z</t>
         </is>
       </c>
     </row>
@@ -28047,7 +28042,7 @@
       </c>
       <c r="P46" t="inlineStr">
         <is>
-          <t>2026-07-25T03:56:46.139Z</t>
+          <t>2026-07-25T04:54:34.143Z</t>
         </is>
       </c>
     </row>
@@ -28117,7 +28112,7 @@
       </c>
       <c r="P47" t="inlineStr">
         <is>
-          <t>2026-07-25T03:57:12.330Z</t>
+          <t>2026-07-25T04:54:34.143Z</t>
         </is>
       </c>
     </row>
@@ -28187,7 +28182,7 @@
       </c>
       <c r="P48" t="inlineStr">
         <is>
-          <t>2026-07-25T03:57:37.841Z</t>
+          <t>2026-07-25T04:54:34.143Z</t>
         </is>
       </c>
     </row>
@@ -28252,7 +28247,7 @@
       </c>
       <c r="P49" t="inlineStr">
         <is>
-          <t>2026-07-25T04:04:26.310Z</t>
+          <t>2026-07-25T04:54:34.143Z</t>
         </is>
       </c>
     </row>
@@ -28322,7 +28317,7 @@
       </c>
       <c r="P50" t="inlineStr">
         <is>
-          <t>2026-07-25T04:04:50.280Z</t>
+          <t>2026-07-25T04:54:34.143Z</t>
         </is>
       </c>
     </row>
@@ -28392,7 +28387,7 @@
       </c>
       <c r="P51" t="inlineStr">
         <is>
-          <t>2026-07-25T04:05:31.707Z</t>
+          <t>2026-07-25T04:54:34.143Z</t>
         </is>
       </c>
     </row>
@@ -28457,7 +28452,7 @@
       </c>
       <c r="P52" t="inlineStr">
         <is>
-          <t>2026-07-25T04:06:06.428Z</t>
+          <t>2026-07-25T04:54:34.143Z</t>
         </is>
       </c>
     </row>
@@ -28527,7 +28522,7 @@
       </c>
       <c r="P53" t="inlineStr">
         <is>
-          <t>2026-07-25T04:06:38.630Z</t>
+          <t>2026-07-25T04:54:34.143Z</t>
         </is>
       </c>
     </row>
@@ -28597,7 +28592,7 @@
       </c>
       <c r="P54" t="inlineStr">
         <is>
-          <t>2026-07-25T04:06:58.252Z</t>
+          <t>2026-07-25T04:54:34.143Z</t>
         </is>
       </c>
     </row>
@@ -28667,7 +28662,7 @@
       </c>
       <c r="P55" t="inlineStr">
         <is>
-          <t>2026-07-25T04:07:19.046Z</t>
+          <t>2026-07-25T04:54:34.143Z</t>
         </is>
       </c>
     </row>
@@ -28737,7 +28732,7 @@
       </c>
       <c r="P56" t="inlineStr">
         <is>
-          <t>2026-07-25T04:08:10.250Z</t>
+          <t>2026-07-25T04:54:34.143Z</t>
         </is>
       </c>
     </row>
@@ -28807,7 +28802,7 @@
       </c>
       <c r="P57" t="inlineStr">
         <is>
-          <t>2026-07-25T04:10:35.995Z</t>
+          <t>2026-07-25T04:54:34.143Z</t>
         </is>
       </c>
     </row>
@@ -28877,7 +28872,7 @@
       </c>
       <c r="P58" t="inlineStr">
         <is>
-          <t>2026-07-25T04:11:17.108Z</t>
+          <t>2026-07-25T04:54:34.143Z</t>
         </is>
       </c>
     </row>
@@ -28892,870 +28887,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D39"/>
+  <dimension ref="A1:A1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="23" customWidth="1" min="1" max="1"/>
-    <col width="39" customWidth="1" min="2" max="2"/>
-    <col width="26" customWidth="1" min="3" max="3"/>
-    <col width="54" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>artist</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>reason</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>recordedAt</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>sourceUrl</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Bakery</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Identity confidence 90% is below 98%.</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>2026-07-25T03:29:12.636Z</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>https://www.lanewaymusic.com.au/bakery</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Bengal Tigers</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Identity confidence 90% is below 98%.</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>2026-07-25T03:29:22.776Z</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>https://www.lanewaymusic.com.au/bengaltigers</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Big Heavy Stuff</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Identity confidence 90% is below 98%.</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>2026-07-25T03:29:34.483Z</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>https://www.lanewaymusic.com.au/big-heavy-stuff</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Blackfeather</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Identity confidence 80% is below 98%.</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>2026-07-25T03:30:46.340Z</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>https://www.lanewaymusic.com.au/blackfeather</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Buzz &amp; The Pickups</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Identity confidence 90% is below 98%.</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>2026-07-25T03:30:55.985Z</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>https://www.lanewaymusic.com.au/buzzandthepickups</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Celibate Rifles</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Identity confidence 80% is below 98%.</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>2026-07-25T03:31:36.755Z</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>https://www.lanewaymusic.com.au/celibaterifles</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>City Sharps</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Identity confidence 80% is below 98%.</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>2026-07-25T03:35:23.359Z</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>https://www.lanewaymusic.com.au/citysharps</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Crash Politics</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Identity confidence 90% is below 98%.</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>2026-07-25T03:35:35.062Z</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>https://www.lanewaymusic.com.au/crashpolitics</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Daniel</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>Identity confidence 80% is below 98%.</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>2026-07-25T03:36:10.422Z</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>https://www.lanewaymusic.com.au/daniel</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Deckchairs Overboard</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>Identity confidence 90% is below 98%.</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>2026-07-25T03:36:44.330Z</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>https://www.lanewaymusic.com.au/deckchairs-overboard</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>Do Re Mi</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>Identity confidence 80% is below 98%.</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>2026-07-25T03:37:12.664Z</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>https://www.lanewaymusic.com.au/do-re-mi</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>Draught Dodgers</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>Identity confidence 80% is below 98%.</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>2026-07-25T03:37:44.098Z</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>https://www.lanewaymusic.com.au/draughtdodgers</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>Eduardo Miller</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>Identity confidence 90% is below 98%.</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>2026-07-25T03:38:14.371Z</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>https://www.lanewaymusic.com.au/eduardo-miller</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>Electric Pandas</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>Identity confidence 80% is below 98%.</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>2026-07-25T03:38:59.808Z</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>https://www.lanewaymusic.com.au/electric-pandas</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>Glyn Mason</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>Identity confidence 80% is below 98%.</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>2026-07-25T03:39:50.483Z</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>https://www.lanewaymusic.com.au/glyn-mason</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>Harem Scarem</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>Identity confidence 90% is below 98%.</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>2026-07-25T03:40:08.143Z</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>https://www.lanewaymusic.com.au/haremscarem</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>James McCann</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>Identity confidence 90% is below 98%.</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>2026-07-25T03:41:10.202Z</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>https://www.lanewaymusic.com.au/jamesmccann</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>Joey Amenta</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>Identity confidence 80% is below 98%.</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>2026-07-25T03:42:44.718Z</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>https://www.lanewaymusic.com.au/joey-amenta</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>Johnny Kannis</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>Identity confidence 90% is below 98%.</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>2026-07-25T03:43:34.419Z</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>https://www.lanewaymusic.com.au/johnny-kannis</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>Kent Steedman</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>Identity confidence 90% is below 98%.</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>2026-07-25T03:44:21.117Z</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>https://www.lanewaymusic.com.au/kentsteedman</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>Mike Rudd</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>Identity confidence 80% is below 98%.</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>2026-07-25T03:49:09.239Z</t>
-        </is>
-      </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>https://www.lanewaymusic.com.au/mike-rudd</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>Mississippi Shakedown</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>Identity confidence 90% is below 98%.</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>2026-07-25T03:49:20.302Z</t>
-        </is>
-      </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>https://www.lanewaymusic.com.au/mississippishakedown</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>New Age</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>Identity confidence 90% is below 98%.</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>2026-07-25T03:49:47.903Z</t>
-        </is>
-      </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>https://www.lanewaymusic.com.au/new-age</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>Old Blue Dogs</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>Identity confidence 90% is below 98%.</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>2026-07-25T03:49:57.214Z</t>
-        </is>
-      </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>https://www.lanewaymusic.com.au/oldbluedogs</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>Phil Manning</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>Identity confidence 90% is below 98%.</t>
-        </is>
-      </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>2026-07-25T03:50:49.599Z</t>
-        </is>
-      </c>
-      <c r="D26" t="inlineStr">
-        <is>
-          <t>https://www.lanewaymusic.com.au/phil-manning</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>Radio KSG</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>Identity confidence 80% is below 98%.</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>2026-07-25T03:54:55.081Z</t>
-        </is>
-      </c>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t>https://www.lanewaymusic.com.au/radioksg</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>ReggaeSPYS</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>Identity confidence 90% is below 98%.</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>2026-07-25T03:55:06.239Z</t>
-        </is>
-      </c>
-      <c r="D28" t="inlineStr">
-        <is>
-          <t>https://www.lanewaymusic.com.au/reggaespys</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>Serelle</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>Identity confidence 80% is below 98%.</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>2026-07-25T03:55:35.577Z</t>
-        </is>
-      </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>https://www.lanewaymusic.com.au/serelle</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>She's The Driver</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>Identity confidence 40% is below 98%.</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>2026-07-25T03:56:08.061Z</t>
-        </is>
-      </c>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>https://www.lanewaymusic.com.au/she-s-the-driver</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>Stephen Walls</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>Identity confidence 80% is below 98%.</t>
-        </is>
-      </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>2026-07-25T03:57:47.136Z</t>
-        </is>
-      </c>
-      <c r="D31" t="inlineStr">
-        <is>
-          <t>https://www.lanewaymusic.com.au/stephenwalls</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>Steve Hoy</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>Identity confidence 80% is below 98%.</t>
-        </is>
-      </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>2026-07-25T03:57:59.333Z</t>
-        </is>
-      </c>
-      <c r="D32" t="inlineStr">
-        <is>
-          <t>https://www.lanewaymusic.com.au/steve-hoy</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>Stockley See Mason</t>
-        </is>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>Identity confidence 80% is below 98%.</t>
-        </is>
-      </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>2026-07-25T03:58:09.188Z</t>
-        </is>
-      </c>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>https://www.lanewaymusic.com.au/stockleyseemason</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>The Hitmen</t>
-        </is>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>Identity confidence 90% is below 98%.</t>
-        </is>
-      </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>2026-07-25T04:05:09.438Z</t>
-        </is>
-      </c>
-      <c r="D34" t="inlineStr">
-        <is>
-          <t>https://www.lanewaymusic.com.au/the-hitmen</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>Them Swoops</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>Identity confidence 90% is below 98%.</t>
-        </is>
-      </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>2026-07-25T04:06:20.666Z</t>
-        </is>
-      </c>
-      <c r="D35" t="inlineStr">
-        <is>
-          <t>https://www.lanewaymusic.com.au/themswoops</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>Vanilla Chainsaws</t>
-        </is>
-      </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>Identity confidence 90% is below 98%.</t>
-        </is>
-      </c>
-      <c r="C36" t="inlineStr">
-        <is>
-          <t>2026-07-25T04:07:30.399Z</t>
-        </is>
-      </c>
-      <c r="D36" t="inlineStr">
-        <is>
-          <t>https://www.lanewaymusic.com.au/vanillachainsaws</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>Violetine</t>
-        </is>
-      </c>
-      <c r="B37" t="inlineStr">
-        <is>
-          <t>Identity confidence 80% is below 98%.</t>
-        </is>
-      </c>
-      <c r="C37" t="inlineStr">
-        <is>
-          <t>2026-07-25T04:07:41.094Z</t>
-        </is>
-      </c>
-      <c r="D37" t="inlineStr">
-        <is>
-          <t>https://www.lanewaymusic.com.au/violetine</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>Young Modern</t>
-        </is>
-      </c>
-      <c r="B38" t="inlineStr">
-        <is>
-          <t>Identity confidence 80% is below 98%.</t>
-        </is>
-      </c>
-      <c r="C38" t="inlineStr">
-        <is>
-          <t>2026-07-25T04:08:24.030Z</t>
-        </is>
-      </c>
-      <c r="D38" t="inlineStr">
-        <is>
-          <t>https://www.lanewaymusic.com.au/youngmodern</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>vSpy vSpy</t>
-        </is>
-      </c>
-      <c r="B39" t="inlineStr">
-        <is>
-          <t>Identity confidence 90% is below 98%.</t>
-        </is>
-      </c>
-      <c r="C39" t="inlineStr">
-        <is>
-          <t>2026-07-25T04:11:34.794Z</t>
-        </is>
-      </c>
-      <c r="D39" t="inlineStr">
-        <is>
-          <t>https://www.lanewaymusic.com.au/v-spy-v-spy</t>
+          <t>No data yet</t>
         </is>
       </c>
     </row>
@@ -29841,7 +28982,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>laneway-music</t>
+          <t>Laneway Music</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -32133,7 +31274,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-07-25T03:28:06.329Z</t>
+          <t>2026-07-25T04:54:16.087Z</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -32186,7 +31327,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2026-07-25T03:28:06.475Z</t>
+          <t>2026-07-25T04:54:16.212Z</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">

</xml_diff>